<commit_message>
Completed CLTV segmentation and business insights
</commit_message>
<xml_diff>
--- a/Output/Customer_CLTV_Analysis.xlsx
+++ b/Output/Customer_CLTV_Analysis.xlsx
@@ -7,7 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Customer_CLTV" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Segment_Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Segment_Behavior" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -424,14 +426,14 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Total_Purchases</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>Total_Revenue</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Total_Purchases</t>
-        </is>
-      </c>
       <c r="D1" t="inlineStr">
         <is>
           <t>Average_Order_Value</t>
@@ -444,12 +446,12 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Customer_Lifetime_Days</t>
+          <t>CLTV</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>CLTV</t>
+          <t>CLTV_Segment</t>
         </is>
       </c>
     </row>
@@ -460,10 +462,10 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
         <v>2175</v>
-      </c>
-      <c r="C2" t="n">
-        <v>1</v>
       </c>
       <c r="D2" t="n">
         <v>2175</v>
@@ -472,10 +474,12 @@
         <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
+        <v>2175</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -485,10 +489,10 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3" t="n">
         <v>2033</v>
-      </c>
-      <c r="C3" t="n">
-        <v>3</v>
       </c>
       <c r="D3" t="n">
         <v>677.67</v>
@@ -497,10 +501,12 @@
         <v>3</v>
       </c>
       <c r="F3" t="n">
-        <v>161</v>
-      </c>
-      <c r="G3" t="n">
-        <v>896.75</v>
+        <v>2033</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -510,10 +516,10 @@
         </is>
       </c>
       <c r="B4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" t="n">
         <v>2165</v>
-      </c>
-      <c r="C4" t="n">
-        <v>4</v>
       </c>
       <c r="D4" t="n">
         <v>541.25</v>
@@ -522,10 +528,12 @@
         <v>4</v>
       </c>
       <c r="F4" t="n">
-        <v>226</v>
-      </c>
-      <c r="G4" t="n">
-        <v>1340.52</v>
+        <v>2165</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -535,10 +543,10 @@
         </is>
       </c>
       <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="n">
         <v>564</v>
-      </c>
-      <c r="C5" t="n">
-        <v>1</v>
       </c>
       <c r="D5" t="n">
         <v>564</v>
@@ -547,10 +555,12 @@
         <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0</v>
+        <v>564</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -560,10 +570,10 @@
         </is>
       </c>
       <c r="B6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" t="n">
         <v>180</v>
-      </c>
-      <c r="C6" t="n">
-        <v>1</v>
       </c>
       <c r="D6" t="n">
         <v>180</v>
@@ -572,10 +582,12 @@
         <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0</v>
+        <v>180</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -585,10 +597,10 @@
         </is>
       </c>
       <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="n">
         <v>1062</v>
-      </c>
-      <c r="C7" t="n">
-        <v>1</v>
       </c>
       <c r="D7" t="n">
         <v>1062</v>
@@ -597,10 +609,12 @@
         <v>1</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0</v>
+        <v>1062</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -610,10 +624,10 @@
         </is>
       </c>
       <c r="B8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" t="n">
         <v>1151</v>
-      </c>
-      <c r="C8" t="n">
-        <v>2</v>
       </c>
       <c r="D8" t="n">
         <v>575.5</v>
@@ -622,10 +636,12 @@
         <v>2</v>
       </c>
       <c r="F8" t="n">
-        <v>201</v>
-      </c>
-      <c r="G8" t="n">
-        <v>633.84</v>
+        <v>1151</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -635,10 +651,10 @@
         </is>
       </c>
       <c r="B9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C9" t="n">
         <v>3877</v>
-      </c>
-      <c r="C9" t="n">
-        <v>3</v>
       </c>
       <c r="D9" t="n">
         <v>1292.33</v>
@@ -647,10 +663,12 @@
         <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>103</v>
-      </c>
-      <c r="G9" t="n">
-        <v>1094.06</v>
+        <v>3877</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -660,10 +678,10 @@
         </is>
       </c>
       <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="n">
         <v>54</v>
-      </c>
-      <c r="C10" t="n">
-        <v>1</v>
       </c>
       <c r="D10" t="n">
         <v>54</v>
@@ -672,10 +690,12 @@
         <v>1</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0</v>
+        <v>54</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -685,10 +705,10 @@
         </is>
       </c>
       <c r="B11" t="n">
+        <v>3</v>
+      </c>
+      <c r="C11" t="n">
         <v>1317</v>
-      </c>
-      <c r="C11" t="n">
-        <v>3</v>
       </c>
       <c r="D11" t="n">
         <v>439</v>
@@ -697,10 +717,12 @@
         <v>3</v>
       </c>
       <c r="F11" t="n">
-        <v>207</v>
-      </c>
-      <c r="G11" t="n">
-        <v>746.9</v>
+        <v>1317</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -710,10 +732,10 @@
         </is>
       </c>
       <c r="B12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" t="n">
         <v>932</v>
-      </c>
-      <c r="C12" t="n">
-        <v>1</v>
       </c>
       <c r="D12" t="n">
         <v>932</v>
@@ -722,10 +744,12 @@
         <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" t="n">
-        <v>0</v>
+        <v>932</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -735,10 +759,10 @@
         </is>
       </c>
       <c r="B13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" t="n">
         <v>2653</v>
-      </c>
-      <c r="C13" t="n">
-        <v>3</v>
       </c>
       <c r="D13" t="n">
         <v>884.33</v>
@@ -747,10 +771,12 @@
         <v>3</v>
       </c>
       <c r="F13" t="n">
-        <v>195</v>
-      </c>
-      <c r="G13" t="n">
-        <v>1417.36</v>
+        <v>2653</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -760,10 +786,10 @@
         </is>
       </c>
       <c r="B14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" t="n">
         <v>1032</v>
-      </c>
-      <c r="C14" t="n">
-        <v>1</v>
       </c>
       <c r="D14" t="n">
         <v>1032</v>
@@ -772,10 +798,12 @@
         <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" t="n">
-        <v>0</v>
+        <v>1032</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -785,10 +813,10 @@
         </is>
       </c>
       <c r="B15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" t="n">
         <v>336</v>
-      </c>
-      <c r="C15" t="n">
-        <v>1</v>
       </c>
       <c r="D15" t="n">
         <v>336</v>
@@ -797,10 +825,12 @@
         <v>1</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" t="n">
-        <v>0</v>
+        <v>336</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -810,10 +840,10 @@
         </is>
       </c>
       <c r="B16" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" t="n">
         <v>3819</v>
-      </c>
-      <c r="C16" t="n">
-        <v>4</v>
       </c>
       <c r="D16" t="n">
         <v>954.75</v>
@@ -822,10 +852,12 @@
         <v>4</v>
       </c>
       <c r="F16" t="n">
-        <v>264</v>
-      </c>
-      <c r="G16" t="n">
-        <v>2762.24</v>
+        <v>3819</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -835,10 +867,10 @@
         </is>
       </c>
       <c r="B17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" t="n">
         <v>1285</v>
-      </c>
-      <c r="C17" t="n">
-        <v>2</v>
       </c>
       <c r="D17" t="n">
         <v>642.5</v>
@@ -847,10 +879,12 @@
         <v>2</v>
       </c>
       <c r="F17" t="n">
-        <v>110</v>
-      </c>
-      <c r="G17" t="n">
-        <v>387.26</v>
+        <v>1285</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -860,10 +894,10 @@
         </is>
       </c>
       <c r="B18" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" t="n">
         <v>232</v>
-      </c>
-      <c r="C18" t="n">
-        <v>1</v>
       </c>
       <c r="D18" t="n">
         <v>232</v>
@@ -872,10 +906,12 @@
         <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" t="n">
-        <v>0</v>
+        <v>232</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -885,10 +921,10 @@
         </is>
       </c>
       <c r="B19" t="n">
+        <v>5</v>
+      </c>
+      <c r="C19" t="n">
         <v>2264</v>
-      </c>
-      <c r="C19" t="n">
-        <v>5</v>
       </c>
       <c r="D19" t="n">
         <v>452.8</v>
@@ -897,10 +933,12 @@
         <v>5</v>
       </c>
       <c r="F19" t="n">
-        <v>300</v>
-      </c>
-      <c r="G19" t="n">
-        <v>1860.82</v>
+        <v>2264</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -910,10 +948,10 @@
         </is>
       </c>
       <c r="B20" t="n">
+        <v>2</v>
+      </c>
+      <c r="C20" t="n">
         <v>1343</v>
-      </c>
-      <c r="C20" t="n">
-        <v>2</v>
       </c>
       <c r="D20" t="n">
         <v>671.5</v>
@@ -922,10 +960,12 @@
         <v>2</v>
       </c>
       <c r="F20" t="n">
-        <v>175</v>
-      </c>
-      <c r="G20" t="n">
-        <v>643.9</v>
+        <v>1343</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -935,10 +975,10 @@
         </is>
       </c>
       <c r="B21" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" t="n">
         <v>2170</v>
-      </c>
-      <c r="C21" t="n">
-        <v>1</v>
       </c>
       <c r="D21" t="n">
         <v>2170</v>
@@ -947,10 +987,12 @@
         <v>1</v>
       </c>
       <c r="F21" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" t="n">
-        <v>0</v>
+        <v>2170</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -960,10 +1002,10 @@
         </is>
       </c>
       <c r="B22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" t="n">
         <v>504</v>
-      </c>
-      <c r="C22" t="n">
-        <v>1</v>
       </c>
       <c r="D22" t="n">
         <v>504</v>
@@ -972,10 +1014,12 @@
         <v>1</v>
       </c>
       <c r="F22" t="n">
-        <v>0</v>
-      </c>
-      <c r="G22" t="n">
-        <v>0</v>
+        <v>504</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="23">
@@ -985,10 +1029,10 @@
         </is>
       </c>
       <c r="B23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C23" t="n">
         <v>164</v>
-      </c>
-      <c r="C23" t="n">
-        <v>2</v>
       </c>
       <c r="D23" t="n">
         <v>82</v>
@@ -997,10 +1041,12 @@
         <v>2</v>
       </c>
       <c r="F23" t="n">
-        <v>130</v>
-      </c>
-      <c r="G23" t="n">
-        <v>58.41</v>
+        <v>164</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -1010,10 +1056,10 @@
         </is>
       </c>
       <c r="B24" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" t="n">
         <v>930</v>
-      </c>
-      <c r="C24" t="n">
-        <v>1</v>
       </c>
       <c r="D24" t="n">
         <v>930</v>
@@ -1022,10 +1068,12 @@
         <v>1</v>
       </c>
       <c r="F24" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" t="n">
-        <v>0</v>
+        <v>930</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -1035,10 +1083,10 @@
         </is>
       </c>
       <c r="B25" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" t="n">
         <v>705</v>
-      </c>
-      <c r="C25" t="n">
-        <v>1</v>
       </c>
       <c r="D25" t="n">
         <v>705</v>
@@ -1047,10 +1095,12 @@
         <v>1</v>
       </c>
       <c r="F25" t="n">
-        <v>0</v>
-      </c>
-      <c r="G25" t="n">
-        <v>0</v>
+        <v>705</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="26">
@@ -1060,10 +1110,10 @@
         </is>
       </c>
       <c r="B26" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" t="n">
         <v>882</v>
-      </c>
-      <c r="C26" t="n">
-        <v>1</v>
       </c>
       <c r="D26" t="n">
         <v>882</v>
@@ -1072,10 +1122,12 @@
         <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>0</v>
-      </c>
-      <c r="G26" t="n">
-        <v>0</v>
+        <v>882</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="27">
@@ -1085,10 +1137,10 @@
         </is>
       </c>
       <c r="B27" t="n">
+        <v>1</v>
+      </c>
+      <c r="C27" t="n">
         <v>692</v>
-      </c>
-      <c r="C27" t="n">
-        <v>1</v>
       </c>
       <c r="D27" t="n">
         <v>692</v>
@@ -1097,10 +1149,12 @@
         <v>1</v>
       </c>
       <c r="F27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G27" t="n">
-        <v>0</v>
+        <v>692</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="28">
@@ -1110,10 +1164,10 @@
         </is>
       </c>
       <c r="B28" t="n">
+        <v>1</v>
+      </c>
+      <c r="C28" t="n">
         <v>255</v>
-      </c>
-      <c r="C28" t="n">
-        <v>1</v>
       </c>
       <c r="D28" t="n">
         <v>255</v>
@@ -1122,10 +1176,12 @@
         <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>0</v>
-      </c>
-      <c r="G28" t="n">
-        <v>0</v>
+        <v>255</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="29">
@@ -1135,10 +1191,10 @@
         </is>
       </c>
       <c r="B29" t="n">
+        <v>1</v>
+      </c>
+      <c r="C29" t="n">
         <v>888</v>
-      </c>
-      <c r="C29" t="n">
-        <v>1</v>
       </c>
       <c r="D29" t="n">
         <v>888</v>
@@ -1147,10 +1203,12 @@
         <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>0</v>
-      </c>
-      <c r="G29" t="n">
-        <v>0</v>
+        <v>888</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -1160,10 +1218,10 @@
         </is>
       </c>
       <c r="B30" t="n">
+        <v>2</v>
+      </c>
+      <c r="C30" t="n">
         <v>954</v>
-      </c>
-      <c r="C30" t="n">
-        <v>2</v>
       </c>
       <c r="D30" t="n">
         <v>477</v>
@@ -1172,10 +1230,12 @@
         <v>2</v>
       </c>
       <c r="F30" t="n">
-        <v>153</v>
-      </c>
-      <c r="G30" t="n">
-        <v>399.9</v>
+        <v>954</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -1185,10 +1245,10 @@
         </is>
       </c>
       <c r="B31" t="n">
+        <v>2</v>
+      </c>
+      <c r="C31" t="n">
         <v>1371</v>
-      </c>
-      <c r="C31" t="n">
-        <v>2</v>
       </c>
       <c r="D31" t="n">
         <v>685.5</v>
@@ -1197,10 +1257,12 @@
         <v>2</v>
       </c>
       <c r="F31" t="n">
-        <v>80</v>
-      </c>
-      <c r="G31" t="n">
-        <v>300.49</v>
+        <v>1371</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="32">
@@ -1210,10 +1272,10 @@
         </is>
       </c>
       <c r="B32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C32" t="n">
         <v>2827</v>
-      </c>
-      <c r="C32" t="n">
-        <v>3</v>
       </c>
       <c r="D32" t="n">
         <v>942.33</v>
@@ -1222,10 +1284,12 @@
         <v>3</v>
       </c>
       <c r="F32" t="n">
-        <v>183</v>
-      </c>
-      <c r="G32" t="n">
-        <v>1417.37</v>
+        <v>2827</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -1235,10 +1299,10 @@
         </is>
       </c>
       <c r="B33" t="n">
+        <v>2</v>
+      </c>
+      <c r="C33" t="n">
         <v>431</v>
-      </c>
-      <c r="C33" t="n">
-        <v>2</v>
       </c>
       <c r="D33" t="n">
         <v>215.5</v>
@@ -1247,10 +1311,12 @@
         <v>2</v>
       </c>
       <c r="F33" t="n">
-        <v>231</v>
-      </c>
-      <c r="G33" t="n">
-        <v>272.77</v>
+        <v>431</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="34">
@@ -1260,10 +1326,10 @@
         </is>
       </c>
       <c r="B34" t="n">
+        <v>2</v>
+      </c>
+      <c r="C34" t="n">
         <v>3259</v>
-      </c>
-      <c r="C34" t="n">
-        <v>2</v>
       </c>
       <c r="D34" t="n">
         <v>1629.5</v>
@@ -1272,10 +1338,12 @@
         <v>2</v>
       </c>
       <c r="F34" t="n">
-        <v>82</v>
-      </c>
-      <c r="G34" t="n">
-        <v>732.16</v>
+        <v>3259</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="35">
@@ -1285,10 +1353,10 @@
         </is>
       </c>
       <c r="B35" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" t="n">
         <v>1383</v>
-      </c>
-      <c r="C35" t="n">
-        <v>1</v>
       </c>
       <c r="D35" t="n">
         <v>1383</v>
@@ -1297,10 +1365,12 @@
         <v>1</v>
       </c>
       <c r="F35" t="n">
-        <v>0</v>
-      </c>
-      <c r="G35" t="n">
-        <v>0</v>
+        <v>1383</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="36">
@@ -1310,10 +1380,10 @@
         </is>
       </c>
       <c r="B36" t="n">
+        <v>2</v>
+      </c>
+      <c r="C36" t="n">
         <v>3062</v>
-      </c>
-      <c r="C36" t="n">
-        <v>2</v>
       </c>
       <c r="D36" t="n">
         <v>1531</v>
@@ -1322,10 +1392,12 @@
         <v>2</v>
       </c>
       <c r="F36" t="n">
-        <v>144</v>
-      </c>
-      <c r="G36" t="n">
-        <v>1208.02</v>
+        <v>3062</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="37">
@@ -1335,10 +1407,10 @@
         </is>
       </c>
       <c r="B37" t="n">
+        <v>4</v>
+      </c>
+      <c r="C37" t="n">
         <v>2360</v>
-      </c>
-      <c r="C37" t="n">
-        <v>4</v>
       </c>
       <c r="D37" t="n">
         <v>590</v>
@@ -1347,10 +1419,12 @@
         <v>4</v>
       </c>
       <c r="F37" t="n">
-        <v>307</v>
-      </c>
-      <c r="G37" t="n">
-        <v>1984.99</v>
+        <v>2360</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="38">
@@ -1360,10 +1434,10 @@
         </is>
       </c>
       <c r="B38" t="n">
+        <v>1</v>
+      </c>
+      <c r="C38" t="n">
         <v>1944</v>
-      </c>
-      <c r="C38" t="n">
-        <v>1</v>
       </c>
       <c r="D38" t="n">
         <v>1944</v>
@@ -1372,10 +1446,12 @@
         <v>1</v>
       </c>
       <c r="F38" t="n">
-        <v>0</v>
-      </c>
-      <c r="G38" t="n">
-        <v>0</v>
+        <v>1944</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="39">
@@ -1385,10 +1461,10 @@
         </is>
       </c>
       <c r="B39" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" t="n">
         <v>34</v>
-      </c>
-      <c r="C39" t="n">
-        <v>1</v>
       </c>
       <c r="D39" t="n">
         <v>34</v>
@@ -1397,10 +1473,12 @@
         <v>1</v>
       </c>
       <c r="F39" t="n">
-        <v>0</v>
-      </c>
-      <c r="G39" t="n">
-        <v>0</v>
+        <v>34</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="40">
@@ -1410,10 +1488,10 @@
         </is>
       </c>
       <c r="B40" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" t="n">
         <v>1920</v>
-      </c>
-      <c r="C40" t="n">
-        <v>1</v>
       </c>
       <c r="D40" t="n">
         <v>1920</v>
@@ -1422,10 +1500,12 @@
         <v>1</v>
       </c>
       <c r="F40" t="n">
-        <v>0</v>
-      </c>
-      <c r="G40" t="n">
-        <v>0</v>
+        <v>1920</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="41">
@@ -1435,10 +1515,10 @@
         </is>
       </c>
       <c r="B41" t="n">
+        <v>3</v>
+      </c>
+      <c r="C41" t="n">
         <v>2201</v>
-      </c>
-      <c r="C41" t="n">
-        <v>3</v>
       </c>
       <c r="D41" t="n">
         <v>733.67</v>
@@ -1447,10 +1527,12 @@
         <v>3</v>
       </c>
       <c r="F41" t="n">
-        <v>30</v>
-      </c>
-      <c r="G41" t="n">
-        <v>180.9</v>
+        <v>2201</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="42">
@@ -1460,10 +1542,10 @@
         </is>
       </c>
       <c r="B42" t="n">
+        <v>2</v>
+      </c>
+      <c r="C42" t="n">
         <v>3165</v>
-      </c>
-      <c r="C42" t="n">
-        <v>2</v>
       </c>
       <c r="D42" t="n">
         <v>1582.5</v>
@@ -1472,10 +1554,12 @@
         <v>2</v>
       </c>
       <c r="F42" t="n">
-        <v>19</v>
-      </c>
-      <c r="G42" t="n">
-        <v>164.75</v>
+        <v>3165</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="43">
@@ -1485,10 +1569,10 @@
         </is>
       </c>
       <c r="B43" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" t="n">
         <v>1375</v>
-      </c>
-      <c r="C43" t="n">
-        <v>1</v>
       </c>
       <c r="D43" t="n">
         <v>1375</v>
@@ -1497,10 +1581,12 @@
         <v>1</v>
       </c>
       <c r="F43" t="n">
-        <v>0</v>
-      </c>
-      <c r="G43" t="n">
-        <v>0</v>
+        <v>1375</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="44">
@@ -1510,10 +1596,10 @@
         </is>
       </c>
       <c r="B44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" t="n">
         <v>856</v>
-      </c>
-      <c r="C44" t="n">
-        <v>1</v>
       </c>
       <c r="D44" t="n">
         <v>856</v>
@@ -1522,10 +1608,12 @@
         <v>1</v>
       </c>
       <c r="F44" t="n">
-        <v>0</v>
-      </c>
-      <c r="G44" t="n">
-        <v>0</v>
+        <v>856</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="45">
@@ -1535,10 +1623,10 @@
         </is>
       </c>
       <c r="B45" t="n">
+        <v>3</v>
+      </c>
+      <c r="C45" t="n">
         <v>1307</v>
-      </c>
-      <c r="C45" t="n">
-        <v>3</v>
       </c>
       <c r="D45" t="n">
         <v>435.67</v>
@@ -1547,10 +1635,12 @@
         <v>3</v>
       </c>
       <c r="F45" t="n">
-        <v>270</v>
-      </c>
-      <c r="G45" t="n">
-        <v>966.8200000000001</v>
+        <v>1307</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="46">
@@ -1560,10 +1650,10 @@
         </is>
       </c>
       <c r="B46" t="n">
+        <v>2</v>
+      </c>
+      <c r="C46" t="n">
         <v>1139</v>
-      </c>
-      <c r="C46" t="n">
-        <v>2</v>
       </c>
       <c r="D46" t="n">
         <v>569.5</v>
@@ -1572,10 +1662,12 @@
         <v>2</v>
       </c>
       <c r="F46" t="n">
-        <v>114</v>
-      </c>
-      <c r="G46" t="n">
-        <v>355.74</v>
+        <v>1139</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="47">
@@ -1585,10 +1677,10 @@
         </is>
       </c>
       <c r="B47" t="n">
+        <v>1</v>
+      </c>
+      <c r="C47" t="n">
         <v>625</v>
-      </c>
-      <c r="C47" t="n">
-        <v>1</v>
       </c>
       <c r="D47" t="n">
         <v>625</v>
@@ -1597,10 +1689,12 @@
         <v>1</v>
       </c>
       <c r="F47" t="n">
-        <v>0</v>
-      </c>
-      <c r="G47" t="n">
-        <v>0</v>
+        <v>625</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="48">
@@ -1610,10 +1704,10 @@
         </is>
       </c>
       <c r="B48" t="n">
+        <v>3</v>
+      </c>
+      <c r="C48" t="n">
         <v>2060</v>
-      </c>
-      <c r="C48" t="n">
-        <v>3</v>
       </c>
       <c r="D48" t="n">
         <v>686.67</v>
@@ -1622,10 +1716,12 @@
         <v>3</v>
       </c>
       <c r="F48" t="n">
-        <v>138</v>
-      </c>
-      <c r="G48" t="n">
-        <v>778.85</v>
+        <v>2060</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="49">
@@ -1635,10 +1731,10 @@
         </is>
       </c>
       <c r="B49" t="n">
+        <v>1</v>
+      </c>
+      <c r="C49" t="n">
         <v>264</v>
-      </c>
-      <c r="C49" t="n">
-        <v>1</v>
       </c>
       <c r="D49" t="n">
         <v>264</v>
@@ -1647,10 +1743,12 @@
         <v>1</v>
       </c>
       <c r="F49" t="n">
-        <v>0</v>
-      </c>
-      <c r="G49" t="n">
-        <v>0</v>
+        <v>264</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="50">
@@ -1660,10 +1758,10 @@
         </is>
       </c>
       <c r="B50" t="n">
+        <v>2</v>
+      </c>
+      <c r="C50" t="n">
         <v>3692</v>
-      </c>
-      <c r="C50" t="n">
-        <v>2</v>
       </c>
       <c r="D50" t="n">
         <v>1846</v>
@@ -1672,10 +1770,12 @@
         <v>2</v>
       </c>
       <c r="F50" t="n">
-        <v>5</v>
-      </c>
-      <c r="G50" t="n">
-        <v>50.58</v>
+        <v>3692</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="51">
@@ -1685,10 +1785,10 @@
         </is>
       </c>
       <c r="B51" t="n">
+        <v>2</v>
+      </c>
+      <c r="C51" t="n">
         <v>2397</v>
-      </c>
-      <c r="C51" t="n">
-        <v>2</v>
       </c>
       <c r="D51" t="n">
         <v>1198.5</v>
@@ -1697,10 +1797,12 @@
         <v>2</v>
       </c>
       <c r="F51" t="n">
-        <v>288</v>
-      </c>
-      <c r="G51" t="n">
-        <v>1891.33</v>
+        <v>2397</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="52">
@@ -1710,10 +1812,10 @@
         </is>
       </c>
       <c r="B52" t="n">
+        <v>4</v>
+      </c>
+      <c r="C52" t="n">
         <v>3064</v>
-      </c>
-      <c r="C52" t="n">
-        <v>4</v>
       </c>
       <c r="D52" t="n">
         <v>766</v>
@@ -1722,10 +1824,12 @@
         <v>4</v>
       </c>
       <c r="F52" t="n">
-        <v>350</v>
-      </c>
-      <c r="G52" t="n">
-        <v>2938.08</v>
+        <v>3064</v>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="53">
@@ -1735,10 +1839,10 @@
         </is>
       </c>
       <c r="B53" t="n">
+        <v>2</v>
+      </c>
+      <c r="C53" t="n">
         <v>2024</v>
-      </c>
-      <c r="C53" t="n">
-        <v>2</v>
       </c>
       <c r="D53" t="n">
         <v>1012</v>
@@ -1747,10 +1851,12 @@
         <v>2</v>
       </c>
       <c r="F53" t="n">
-        <v>68</v>
-      </c>
-      <c r="G53" t="n">
-        <v>377.07</v>
+        <v>2024</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="54">
@@ -1760,10 +1866,10 @@
         </is>
       </c>
       <c r="B54" t="n">
+        <v>1</v>
+      </c>
+      <c r="C54" t="n">
         <v>310</v>
-      </c>
-      <c r="C54" t="n">
-        <v>1</v>
       </c>
       <c r="D54" t="n">
         <v>310</v>
@@ -1772,10 +1878,12 @@
         <v>1</v>
       </c>
       <c r="F54" t="n">
-        <v>0</v>
-      </c>
-      <c r="G54" t="n">
-        <v>0</v>
+        <v>310</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="55">
@@ -1785,10 +1893,10 @@
         </is>
       </c>
       <c r="B55" t="n">
+        <v>2</v>
+      </c>
+      <c r="C55" t="n">
         <v>215</v>
-      </c>
-      <c r="C55" t="n">
-        <v>2</v>
       </c>
       <c r="D55" t="n">
         <v>107.5</v>
@@ -1797,10 +1905,12 @@
         <v>2</v>
       </c>
       <c r="F55" t="n">
-        <v>129</v>
-      </c>
-      <c r="G55" t="n">
-        <v>75.98999999999999</v>
+        <v>215</v>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="56">
@@ -1810,10 +1920,10 @@
         </is>
       </c>
       <c r="B56" t="n">
+        <v>2</v>
+      </c>
+      <c r="C56" t="n">
         <v>1735</v>
-      </c>
-      <c r="C56" t="n">
-        <v>2</v>
       </c>
       <c r="D56" t="n">
         <v>867.5</v>
@@ -1822,10 +1932,12 @@
         <v>2</v>
       </c>
       <c r="F56" t="n">
-        <v>158</v>
-      </c>
-      <c r="G56" t="n">
-        <v>751.04</v>
+        <v>1735</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="57">
@@ -1835,10 +1947,10 @@
         </is>
       </c>
       <c r="B57" t="n">
+        <v>2</v>
+      </c>
+      <c r="C57" t="n">
         <v>1238</v>
-      </c>
-      <c r="C57" t="n">
-        <v>2</v>
       </c>
       <c r="D57" t="n">
         <v>619</v>
@@ -1847,10 +1959,12 @@
         <v>2</v>
       </c>
       <c r="F57" t="n">
-        <v>37</v>
-      </c>
-      <c r="G57" t="n">
-        <v>125.5</v>
+        <v>1238</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="58">
@@ -1860,10 +1974,10 @@
         </is>
       </c>
       <c r="B58" t="n">
+        <v>2</v>
+      </c>
+      <c r="C58" t="n">
         <v>775</v>
-      </c>
-      <c r="C58" t="n">
-        <v>2</v>
       </c>
       <c r="D58" t="n">
         <v>387.5</v>
@@ -1872,10 +1986,12 @@
         <v>2</v>
       </c>
       <c r="F58" t="n">
-        <v>69</v>
-      </c>
-      <c r="G58" t="n">
-        <v>146.51</v>
+        <v>775</v>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="59">
@@ -1885,10 +2001,10 @@
         </is>
       </c>
       <c r="B59" t="n">
+        <v>1</v>
+      </c>
+      <c r="C59" t="n">
         <v>2400</v>
-      </c>
-      <c r="C59" t="n">
-        <v>1</v>
       </c>
       <c r="D59" t="n">
         <v>2400</v>
@@ -1897,10 +2013,12 @@
         <v>1</v>
       </c>
       <c r="F59" t="n">
-        <v>0</v>
-      </c>
-      <c r="G59" t="n">
-        <v>0</v>
+        <v>2400</v>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="60">
@@ -1910,10 +2028,10 @@
         </is>
       </c>
       <c r="B60" t="n">
+        <v>2</v>
+      </c>
+      <c r="C60" t="n">
         <v>816</v>
-      </c>
-      <c r="C60" t="n">
-        <v>2</v>
       </c>
       <c r="D60" t="n">
         <v>408</v>
@@ -1922,10 +2040,12 @@
         <v>2</v>
       </c>
       <c r="F60" t="n">
-        <v>44</v>
-      </c>
-      <c r="G60" t="n">
-        <v>98.37</v>
+        <v>816</v>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="61">
@@ -1935,10 +2055,10 @@
         </is>
       </c>
       <c r="B61" t="n">
+        <v>2</v>
+      </c>
+      <c r="C61" t="n">
         <v>1365</v>
-      </c>
-      <c r="C61" t="n">
-        <v>2</v>
       </c>
       <c r="D61" t="n">
         <v>682.5</v>
@@ -1947,10 +2067,12 @@
         <v>2</v>
       </c>
       <c r="F61" t="n">
-        <v>323</v>
-      </c>
-      <c r="G61" t="n">
-        <v>1207.93</v>
+        <v>1365</v>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="62">
@@ -1960,10 +2082,10 @@
         </is>
       </c>
       <c r="B62" t="n">
+        <v>2</v>
+      </c>
+      <c r="C62" t="n">
         <v>899</v>
-      </c>
-      <c r="C62" t="n">
-        <v>2</v>
       </c>
       <c r="D62" t="n">
         <v>449.5</v>
@@ -1972,10 +2094,12 @@
         <v>2</v>
       </c>
       <c r="F62" t="n">
-        <v>36</v>
-      </c>
-      <c r="G62" t="n">
-        <v>88.67</v>
+        <v>899</v>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="63">
@@ -1985,10 +2109,10 @@
         </is>
       </c>
       <c r="B63" t="n">
+        <v>1</v>
+      </c>
+      <c r="C63" t="n">
         <v>36</v>
-      </c>
-      <c r="C63" t="n">
-        <v>1</v>
       </c>
       <c r="D63" t="n">
         <v>36</v>
@@ -1997,10 +2121,12 @@
         <v>1</v>
       </c>
       <c r="F63" t="n">
-        <v>0</v>
-      </c>
-      <c r="G63" t="n">
-        <v>0</v>
+        <v>36</v>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="64">
@@ -2010,10 +2136,10 @@
         </is>
       </c>
       <c r="B64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C64" t="n">
         <v>1875</v>
-      </c>
-      <c r="C64" t="n">
-        <v>1</v>
       </c>
       <c r="D64" t="n">
         <v>1875</v>
@@ -2022,10 +2148,12 @@
         <v>1</v>
       </c>
       <c r="F64" t="n">
-        <v>0</v>
-      </c>
-      <c r="G64" t="n">
-        <v>0</v>
+        <v>1875</v>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="65">
@@ -2035,10 +2163,10 @@
         </is>
       </c>
       <c r="B65" t="n">
+        <v>2</v>
+      </c>
+      <c r="C65" t="n">
         <v>549</v>
-      </c>
-      <c r="C65" t="n">
-        <v>2</v>
       </c>
       <c r="D65" t="n">
         <v>274.5</v>
@@ -2047,10 +2175,12 @@
         <v>2</v>
       </c>
       <c r="F65" t="n">
-        <v>3</v>
-      </c>
-      <c r="G65" t="n">
-        <v>4.51</v>
+        <v>549</v>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="66">
@@ -2060,10 +2190,10 @@
         </is>
       </c>
       <c r="B66" t="n">
+        <v>2</v>
+      </c>
+      <c r="C66" t="n">
         <v>2839</v>
-      </c>
-      <c r="C66" t="n">
-        <v>2</v>
       </c>
       <c r="D66" t="n">
         <v>1419.5</v>
@@ -2072,10 +2202,12 @@
         <v>2</v>
       </c>
       <c r="F66" t="n">
-        <v>75</v>
-      </c>
-      <c r="G66" t="n">
-        <v>583.36</v>
+        <v>2839</v>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="67">
@@ -2085,10 +2217,10 @@
         </is>
       </c>
       <c r="B67" t="n">
+        <v>2</v>
+      </c>
+      <c r="C67" t="n">
         <v>1949</v>
-      </c>
-      <c r="C67" t="n">
-        <v>2</v>
       </c>
       <c r="D67" t="n">
         <v>974.5</v>
@@ -2097,10 +2229,12 @@
         <v>2</v>
       </c>
       <c r="F67" t="n">
-        <v>58</v>
-      </c>
-      <c r="G67" t="n">
-        <v>309.7</v>
+        <v>1949</v>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="68">
@@ -2110,10 +2244,10 @@
         </is>
       </c>
       <c r="B68" t="n">
+        <v>1</v>
+      </c>
+      <c r="C68" t="n">
         <v>95</v>
-      </c>
-      <c r="C68" t="n">
-        <v>1</v>
       </c>
       <c r="D68" t="n">
         <v>95</v>
@@ -2122,10 +2256,12 @@
         <v>1</v>
       </c>
       <c r="F68" t="n">
-        <v>0</v>
-      </c>
-      <c r="G68" t="n">
-        <v>0</v>
+        <v>95</v>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="69">
@@ -2135,10 +2271,10 @@
         </is>
       </c>
       <c r="B69" t="n">
+        <v>2</v>
+      </c>
+      <c r="C69" t="n">
         <v>3209</v>
-      </c>
-      <c r="C69" t="n">
-        <v>2</v>
       </c>
       <c r="D69" t="n">
         <v>1604.5</v>
@@ -2147,10 +2283,12 @@
         <v>2</v>
       </c>
       <c r="F69" t="n">
-        <v>182</v>
-      </c>
-      <c r="G69" t="n">
-        <v>1600.1</v>
+        <v>3209</v>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="70">
@@ -2160,10 +2298,10 @@
         </is>
       </c>
       <c r="B70" t="n">
+        <v>1</v>
+      </c>
+      <c r="C70" t="n">
         <v>86</v>
-      </c>
-      <c r="C70" t="n">
-        <v>1</v>
       </c>
       <c r="D70" t="n">
         <v>86</v>
@@ -2172,10 +2310,12 @@
         <v>1</v>
       </c>
       <c r="F70" t="n">
-        <v>0</v>
-      </c>
-      <c r="G70" t="n">
-        <v>0</v>
+        <v>86</v>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="71">
@@ -2185,10 +2325,10 @@
         </is>
       </c>
       <c r="B71" t="n">
+        <v>1</v>
+      </c>
+      <c r="C71" t="n">
         <v>1284</v>
-      </c>
-      <c r="C71" t="n">
-        <v>1</v>
       </c>
       <c r="D71" t="n">
         <v>1284</v>
@@ -2197,10 +2337,12 @@
         <v>1</v>
       </c>
       <c r="F71" t="n">
-        <v>0</v>
-      </c>
-      <c r="G71" t="n">
-        <v>0</v>
+        <v>1284</v>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="72">
@@ -2210,10 +2352,10 @@
         </is>
       </c>
       <c r="B72" t="n">
+        <v>4</v>
+      </c>
+      <c r="C72" t="n">
         <v>4018</v>
-      </c>
-      <c r="C72" t="n">
-        <v>4</v>
       </c>
       <c r="D72" t="n">
         <v>1004.5</v>
@@ -2222,10 +2364,12 @@
         <v>4</v>
       </c>
       <c r="F72" t="n">
-        <v>191</v>
-      </c>
-      <c r="G72" t="n">
-        <v>2102.57</v>
+        <v>4018</v>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="73">
@@ -2235,10 +2379,10 @@
         </is>
       </c>
       <c r="B73" t="n">
+        <v>1</v>
+      </c>
+      <c r="C73" t="n">
         <v>702</v>
-      </c>
-      <c r="C73" t="n">
-        <v>1</v>
       </c>
       <c r="D73" t="n">
         <v>702</v>
@@ -2247,10 +2391,12 @@
         <v>1</v>
       </c>
       <c r="F73" t="n">
-        <v>0</v>
-      </c>
-      <c r="G73" t="n">
-        <v>0</v>
+        <v>702</v>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="74">
@@ -2260,10 +2406,10 @@
         </is>
       </c>
       <c r="B74" t="n">
+        <v>6</v>
+      </c>
+      <c r="C74" t="n">
         <v>5644</v>
-      </c>
-      <c r="C74" t="n">
-        <v>6</v>
       </c>
       <c r="D74" t="n">
         <v>940.67</v>
@@ -2272,10 +2418,12 @@
         <v>6</v>
       </c>
       <c r="F74" t="n">
-        <v>288</v>
-      </c>
-      <c r="G74" t="n">
-        <v>4453.35</v>
+        <v>5644</v>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="75">
@@ -2285,10 +2433,10 @@
         </is>
       </c>
       <c r="B75" t="n">
+        <v>1</v>
+      </c>
+      <c r="C75" t="n">
         <v>153</v>
-      </c>
-      <c r="C75" t="n">
-        <v>1</v>
       </c>
       <c r="D75" t="n">
         <v>153</v>
@@ -2297,10 +2445,12 @@
         <v>1</v>
       </c>
       <c r="F75" t="n">
-        <v>0</v>
-      </c>
-      <c r="G75" t="n">
-        <v>0</v>
+        <v>153</v>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="76">
@@ -2310,10 +2460,10 @@
         </is>
       </c>
       <c r="B76" t="n">
+        <v>1</v>
+      </c>
+      <c r="C76" t="n">
         <v>816</v>
-      </c>
-      <c r="C76" t="n">
-        <v>1</v>
       </c>
       <c r="D76" t="n">
         <v>816</v>
@@ -2322,10 +2472,12 @@
         <v>1</v>
       </c>
       <c r="F76" t="n">
-        <v>0</v>
-      </c>
-      <c r="G76" t="n">
-        <v>0</v>
+        <v>816</v>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="77">
@@ -2335,10 +2487,10 @@
         </is>
       </c>
       <c r="B77" t="n">
+        <v>5</v>
+      </c>
+      <c r="C77" t="n">
         <v>5266</v>
-      </c>
-      <c r="C77" t="n">
-        <v>5</v>
       </c>
       <c r="D77" t="n">
         <v>1053.2</v>
@@ -2347,10 +2499,12 @@
         <v>5</v>
       </c>
       <c r="F77" t="n">
-        <v>200</v>
-      </c>
-      <c r="G77" t="n">
-        <v>2885.48</v>
+        <v>5266</v>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="78">
@@ -2360,10 +2514,10 @@
         </is>
       </c>
       <c r="B78" t="n">
+        <v>2</v>
+      </c>
+      <c r="C78" t="n">
         <v>1438</v>
-      </c>
-      <c r="C78" t="n">
-        <v>2</v>
       </c>
       <c r="D78" t="n">
         <v>719</v>
@@ -2372,10 +2526,12 @@
         <v>2</v>
       </c>
       <c r="F78" t="n">
-        <v>125</v>
-      </c>
-      <c r="G78" t="n">
-        <v>492.47</v>
+        <v>1438</v>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="79">
@@ -2385,10 +2541,10 @@
         </is>
       </c>
       <c r="B79" t="n">
+        <v>4</v>
+      </c>
+      <c r="C79" t="n">
         <v>2383</v>
-      </c>
-      <c r="C79" t="n">
-        <v>4</v>
       </c>
       <c r="D79" t="n">
         <v>595.75</v>
@@ -2397,10 +2553,12 @@
         <v>4</v>
       </c>
       <c r="F79" t="n">
-        <v>107</v>
-      </c>
-      <c r="G79" t="n">
-        <v>698.58</v>
+        <v>2383</v>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="80">
@@ -2410,10 +2568,10 @@
         </is>
       </c>
       <c r="B80" t="n">
+        <v>4</v>
+      </c>
+      <c r="C80" t="n">
         <v>2883</v>
-      </c>
-      <c r="C80" t="n">
-        <v>4</v>
       </c>
       <c r="D80" t="n">
         <v>720.75</v>
@@ -2422,10 +2580,12 @@
         <v>4</v>
       </c>
       <c r="F80" t="n">
-        <v>255</v>
-      </c>
-      <c r="G80" t="n">
-        <v>2014.15</v>
+        <v>2883</v>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="81">
@@ -2435,10 +2595,10 @@
         </is>
       </c>
       <c r="B81" t="n">
+        <v>1</v>
+      </c>
+      <c r="C81" t="n">
         <v>85</v>
-      </c>
-      <c r="C81" t="n">
-        <v>1</v>
       </c>
       <c r="D81" t="n">
         <v>85</v>
@@ -2447,10 +2607,12 @@
         <v>1</v>
       </c>
       <c r="F81" t="n">
-        <v>0</v>
-      </c>
-      <c r="G81" t="n">
-        <v>0</v>
+        <v>85</v>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="82">
@@ -2460,10 +2622,10 @@
         </is>
       </c>
       <c r="B82" t="n">
+        <v>1</v>
+      </c>
+      <c r="C82" t="n">
         <v>1125</v>
-      </c>
-      <c r="C82" t="n">
-        <v>1</v>
       </c>
       <c r="D82" t="n">
         <v>1125</v>
@@ -2472,10 +2634,12 @@
         <v>1</v>
       </c>
       <c r="F82" t="n">
-        <v>0</v>
-      </c>
-      <c r="G82" t="n">
-        <v>0</v>
+        <v>1125</v>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="83">
@@ -2485,10 +2649,10 @@
         </is>
       </c>
       <c r="B83" t="n">
+        <v>4</v>
+      </c>
+      <c r="C83" t="n">
         <v>3570</v>
-      </c>
-      <c r="C83" t="n">
-        <v>4</v>
       </c>
       <c r="D83" t="n">
         <v>892.5</v>
@@ -2497,10 +2661,12 @@
         <v>4</v>
       </c>
       <c r="F83" t="n">
-        <v>272</v>
-      </c>
-      <c r="G83" t="n">
-        <v>2660.38</v>
+        <v>3570</v>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="84">
@@ -2510,10 +2676,10 @@
         </is>
       </c>
       <c r="B84" t="n">
+        <v>2</v>
+      </c>
+      <c r="C84" t="n">
         <v>1744</v>
-      </c>
-      <c r="C84" t="n">
-        <v>2</v>
       </c>
       <c r="D84" t="n">
         <v>872</v>
@@ -2522,10 +2688,12 @@
         <v>2</v>
       </c>
       <c r="F84" t="n">
-        <v>33</v>
-      </c>
-      <c r="G84" t="n">
-        <v>157.68</v>
+        <v>1744</v>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="85">
@@ -2535,10 +2703,10 @@
         </is>
       </c>
       <c r="B85" t="n">
+        <v>2</v>
+      </c>
+      <c r="C85" t="n">
         <v>388</v>
-      </c>
-      <c r="C85" t="n">
-        <v>2</v>
       </c>
       <c r="D85" t="n">
         <v>194</v>
@@ -2547,10 +2715,12 @@
         <v>2</v>
       </c>
       <c r="F85" t="n">
-        <v>88</v>
-      </c>
-      <c r="G85" t="n">
-        <v>93.55</v>
+        <v>388</v>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="86">
@@ -2560,10 +2730,10 @@
         </is>
       </c>
       <c r="B86" t="n">
+        <v>1</v>
+      </c>
+      <c r="C86" t="n">
         <v>858</v>
-      </c>
-      <c r="C86" t="n">
-        <v>1</v>
       </c>
       <c r="D86" t="n">
         <v>858</v>
@@ -2572,10 +2742,12 @@
         <v>1</v>
       </c>
       <c r="F86" t="n">
-        <v>0</v>
-      </c>
-      <c r="G86" t="n">
-        <v>0</v>
+        <v>858</v>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="87">
@@ -2585,10 +2757,10 @@
         </is>
       </c>
       <c r="B87" t="n">
+        <v>2</v>
+      </c>
+      <c r="C87" t="n">
         <v>678</v>
-      </c>
-      <c r="C87" t="n">
-        <v>2</v>
       </c>
       <c r="D87" t="n">
         <v>339</v>
@@ -2597,10 +2769,12 @@
         <v>2</v>
       </c>
       <c r="F87" t="n">
-        <v>116</v>
-      </c>
-      <c r="G87" t="n">
-        <v>215.47</v>
+        <v>678</v>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="88">
@@ -2610,10 +2784,10 @@
         </is>
       </c>
       <c r="B88" t="n">
+        <v>2</v>
+      </c>
+      <c r="C88" t="n">
         <v>806</v>
-      </c>
-      <c r="C88" t="n">
-        <v>2</v>
       </c>
       <c r="D88" t="n">
         <v>403</v>
@@ -2622,10 +2796,12 @@
         <v>2</v>
       </c>
       <c r="F88" t="n">
-        <v>44</v>
-      </c>
-      <c r="G88" t="n">
-        <v>97.16</v>
+        <v>806</v>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="89">
@@ -2635,10 +2811,10 @@
         </is>
       </c>
       <c r="B89" t="n">
+        <v>1</v>
+      </c>
+      <c r="C89" t="n">
         <v>391</v>
-      </c>
-      <c r="C89" t="n">
-        <v>1</v>
       </c>
       <c r="D89" t="n">
         <v>391</v>
@@ -2647,10 +2823,12 @@
         <v>1</v>
       </c>
       <c r="F89" t="n">
-        <v>0</v>
-      </c>
-      <c r="G89" t="n">
-        <v>0</v>
+        <v>391</v>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="90">
@@ -2660,10 +2838,10 @@
         </is>
       </c>
       <c r="B90" t="n">
+        <v>1</v>
+      </c>
+      <c r="C90" t="n">
         <v>288</v>
-      </c>
-      <c r="C90" t="n">
-        <v>1</v>
       </c>
       <c r="D90" t="n">
         <v>288</v>
@@ -2672,10 +2850,12 @@
         <v>1</v>
       </c>
       <c r="F90" t="n">
-        <v>0</v>
-      </c>
-      <c r="G90" t="n">
-        <v>0</v>
+        <v>288</v>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="91">
@@ -2685,10 +2865,10 @@
         </is>
       </c>
       <c r="B91" t="n">
+        <v>1</v>
+      </c>
+      <c r="C91" t="n">
         <v>864</v>
-      </c>
-      <c r="C91" t="n">
-        <v>1</v>
       </c>
       <c r="D91" t="n">
         <v>864</v>
@@ -2697,10 +2877,12 @@
         <v>1</v>
       </c>
       <c r="F91" t="n">
-        <v>0</v>
-      </c>
-      <c r="G91" t="n">
-        <v>0</v>
+        <v>864</v>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="92">
@@ -2710,10 +2892,10 @@
         </is>
       </c>
       <c r="B92" t="n">
+        <v>1</v>
+      </c>
+      <c r="C92" t="n">
         <v>270</v>
-      </c>
-      <c r="C92" t="n">
-        <v>1</v>
       </c>
       <c r="D92" t="n">
         <v>270</v>
@@ -2722,10 +2904,12 @@
         <v>1</v>
       </c>
       <c r="F92" t="n">
-        <v>0</v>
-      </c>
-      <c r="G92" t="n">
-        <v>0</v>
+        <v>270</v>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="93">
@@ -2735,10 +2919,10 @@
         </is>
       </c>
       <c r="B93" t="n">
+        <v>2</v>
+      </c>
+      <c r="C93" t="n">
         <v>2380</v>
-      </c>
-      <c r="C93" t="n">
-        <v>2</v>
       </c>
       <c r="D93" t="n">
         <v>1190</v>
@@ -2747,10 +2931,12 @@
         <v>2</v>
       </c>
       <c r="F93" t="n">
-        <v>215</v>
-      </c>
-      <c r="G93" t="n">
-        <v>1401.92</v>
+        <v>2380</v>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="94">
@@ -2760,10 +2946,10 @@
         </is>
       </c>
       <c r="B94" t="n">
+        <v>3</v>
+      </c>
+      <c r="C94" t="n">
         <v>2113</v>
-      </c>
-      <c r="C94" t="n">
-        <v>3</v>
       </c>
       <c r="D94" t="n">
         <v>704.33</v>
@@ -2772,10 +2958,12 @@
         <v>3</v>
       </c>
       <c r="F94" t="n">
-        <v>188</v>
-      </c>
-      <c r="G94" t="n">
-        <v>1088.34</v>
+        <v>2113</v>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="95">
@@ -2785,10 +2973,10 @@
         </is>
       </c>
       <c r="B95" t="n">
+        <v>1</v>
+      </c>
+      <c r="C95" t="n">
         <v>1404</v>
-      </c>
-      <c r="C95" t="n">
-        <v>1</v>
       </c>
       <c r="D95" t="n">
         <v>1404</v>
@@ -2797,10 +2985,12 @@
         <v>1</v>
       </c>
       <c r="F95" t="n">
-        <v>0</v>
-      </c>
-      <c r="G95" t="n">
-        <v>0</v>
+        <v>1404</v>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="96">
@@ -2810,10 +3000,10 @@
         </is>
       </c>
       <c r="B96" t="n">
+        <v>2</v>
+      </c>
+      <c r="C96" t="n">
         <v>487</v>
-      </c>
-      <c r="C96" t="n">
-        <v>2</v>
       </c>
       <c r="D96" t="n">
         <v>243.5</v>
@@ -2822,10 +3012,12 @@
         <v>2</v>
       </c>
       <c r="F96" t="n">
-        <v>66</v>
-      </c>
-      <c r="G96" t="n">
-        <v>88.06</v>
+        <v>487</v>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="97">
@@ -2835,10 +3027,10 @@
         </is>
       </c>
       <c r="B97" t="n">
+        <v>2</v>
+      </c>
+      <c r="C97" t="n">
         <v>962</v>
-      </c>
-      <c r="C97" t="n">
-        <v>2</v>
       </c>
       <c r="D97" t="n">
         <v>481</v>
@@ -2847,10 +3039,12 @@
         <v>2</v>
       </c>
       <c r="F97" t="n">
-        <v>40</v>
-      </c>
-      <c r="G97" t="n">
-        <v>105.42</v>
+        <v>962</v>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="98">
@@ -2860,10 +3054,10 @@
         </is>
       </c>
       <c r="B98" t="n">
+        <v>3</v>
+      </c>
+      <c r="C98" t="n">
         <v>3493</v>
-      </c>
-      <c r="C98" t="n">
-        <v>3</v>
       </c>
       <c r="D98" t="n">
         <v>1164.33</v>
@@ -2872,10 +3066,12 @@
         <v>3</v>
       </c>
       <c r="F98" t="n">
-        <v>208</v>
-      </c>
-      <c r="G98" t="n">
-        <v>1990.53</v>
+        <v>3493</v>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="99">
@@ -2885,10 +3081,10 @@
         </is>
       </c>
       <c r="B99" t="n">
+        <v>1</v>
+      </c>
+      <c r="C99" t="n">
         <v>951</v>
-      </c>
-      <c r="C99" t="n">
-        <v>1</v>
       </c>
       <c r="D99" t="n">
         <v>951</v>
@@ -2897,10 +3093,12 @@
         <v>1</v>
       </c>
       <c r="F99" t="n">
-        <v>0</v>
-      </c>
-      <c r="G99" t="n">
-        <v>0</v>
+        <v>951</v>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="100">
@@ -2910,10 +3108,10 @@
         </is>
       </c>
       <c r="B100" t="n">
+        <v>2</v>
+      </c>
+      <c r="C100" t="n">
         <v>450</v>
-      </c>
-      <c r="C100" t="n">
-        <v>2</v>
       </c>
       <c r="D100" t="n">
         <v>225</v>
@@ -2922,10 +3120,12 @@
         <v>2</v>
       </c>
       <c r="F100" t="n">
-        <v>1</v>
-      </c>
-      <c r="G100" t="n">
-        <v>1.23</v>
+        <v>450</v>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="101">
@@ -2935,10 +3135,10 @@
         </is>
       </c>
       <c r="B101" t="n">
+        <v>1</v>
+      </c>
+      <c r="C101" t="n">
         <v>366</v>
-      </c>
-      <c r="C101" t="n">
-        <v>1</v>
       </c>
       <c r="D101" t="n">
         <v>366</v>
@@ -2947,10 +3147,12 @@
         <v>1</v>
       </c>
       <c r="F101" t="n">
-        <v>0</v>
-      </c>
-      <c r="G101" t="n">
-        <v>0</v>
+        <v>366</v>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="102">
@@ -2960,10 +3162,10 @@
         </is>
       </c>
       <c r="B102" t="n">
+        <v>3</v>
+      </c>
+      <c r="C102" t="n">
         <v>1554</v>
-      </c>
-      <c r="C102" t="n">
-        <v>3</v>
       </c>
       <c r="D102" t="n">
         <v>518</v>
@@ -2972,10 +3174,12 @@
         <v>3</v>
       </c>
       <c r="F102" t="n">
-        <v>94</v>
-      </c>
-      <c r="G102" t="n">
-        <v>400.21</v>
+        <v>1554</v>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
       </c>
     </row>
     <row r="103">
@@ -2985,10 +3189,10 @@
         </is>
       </c>
       <c r="B103" t="n">
+        <v>2</v>
+      </c>
+      <c r="C103" t="n">
         <v>3192</v>
-      </c>
-      <c r="C103" t="n">
-        <v>2</v>
       </c>
       <c r="D103" t="n">
         <v>1596</v>
@@ -2997,10 +3201,12 @@
         <v>2</v>
       </c>
       <c r="F103" t="n">
-        <v>95</v>
-      </c>
-      <c r="G103" t="n">
-        <v>830.79</v>
+        <v>3192</v>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="104">
@@ -3010,10 +3216,10 @@
         </is>
       </c>
       <c r="B104" t="n">
+        <v>2</v>
+      </c>
+      <c r="C104" t="n">
         <v>2101</v>
-      </c>
-      <c r="C104" t="n">
-        <v>2</v>
       </c>
       <c r="D104" t="n">
         <v>1050.5</v>
@@ -3022,10 +3228,12 @@
         <v>2</v>
       </c>
       <c r="F104" t="n">
-        <v>1</v>
-      </c>
-      <c r="G104" t="n">
-        <v>5.76</v>
+        <v>2101</v>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
       </c>
     </row>
     <row r="105">
@@ -3035,10 +3243,10 @@
         </is>
       </c>
       <c r="B105" t="n">
+        <v>1</v>
+      </c>
+      <c r="C105" t="n">
         <v>708</v>
-      </c>
-      <c r="C105" t="n">
-        <v>1</v>
       </c>
       <c r="D105" t="n">
         <v>708</v>
@@ -3047,10 +3255,12 @@
         <v>1</v>
       </c>
       <c r="F105" t="n">
-        <v>0</v>
-      </c>
-      <c r="G105" t="n">
-        <v>0</v>
+        <v>708</v>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
       </c>
     </row>
     <row r="106">
@@ -3060,10 +3270,10 @@
         </is>
       </c>
       <c r="B106" t="n">
+        <v>1</v>
+      </c>
+      <c r="C106" t="n">
         <v>198</v>
-      </c>
-      <c r="C106" t="n">
-        <v>1</v>
       </c>
       <c r="D106" t="n">
         <v>198</v>
@@ -3072,10 +3282,180 @@
         <v>1</v>
       </c>
       <c r="F106" t="n">
-        <v>0</v>
-      </c>
-      <c r="G106" t="n">
-        <v>0</v>
+        <v>198</v>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>CLTV_Segment</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Customer_Count</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Average_CLTV</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Total_Revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>35</v>
+      </c>
+      <c r="C2" t="n">
+        <v>373.6</v>
+      </c>
+      <c r="D2" t="n">
+        <v>13076</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>35</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1201.57</v>
+      </c>
+      <c r="D3" t="n">
+        <v>42055</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>35</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2875.74</v>
+      </c>
+      <c r="D4" t="n">
+        <v>100651</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>CLTV_Segment</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Avg_Purchases</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Avg_Order_Value</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Avg_Revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="C2" t="n">
+        <v>302.99</v>
+      </c>
+      <c r="D2" t="n">
+        <v>373.6</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1.57</v>
+      </c>
+      <c r="C3" t="n">
+        <v>872.85</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1201.57</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2.86</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1169.18</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2875.74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>